<commit_message>
chore: add coverage and fix some issues
</commit_message>
<xml_diff>
--- a/src/test/resources/mock/test-bad-student-grade-import.xlsx
+++ b/src/test/resources/mock/test-bad-student-grade-import.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
   <si>
     <t>ref</t>
   </si>
@@ -184,6 +184,12 @@
   </si>
   <si>
     <t>STD0054-XLSX</t>
+  </si>
+  <si>
+    <t>string</t>
+  </si>
+  <si>
+    <t>23001STD</t>
   </si>
 </sst>
 </file>
@@ -1166,23 +1172,30 @@
         <v>55</v>
       </c>
       <c r="B55" s="2">
-        <v>7.5</v>
+        <f>SUM(B53:B54)</f>
+        <v>16.5</v>
       </c>
     </row>
     <row r="56" ht="14.25">
       <c r="A56" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B56" s="2">
-        <v>7</v>
+      <c r="B56" s="2" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="57" ht="14.25">
+      <c r="A57" t="s">
+        <v>57</v>
+      </c>
       <c r="B57" s="2">
         <v>6.5</v>
       </c>
     </row>
     <row r="58" ht="14.25">
+      <c r="A58" s="2" t="s">
+        <v>55</v>
+      </c>
       <c r="B58" s="2">
         <v>6</v>
       </c>

</xml_diff>